<commit_message>
Fixed 1500 and salary conflict
</commit_message>
<xml_diff>
--- a/instruction_data/templates/dec_final/PIT_SI.xlsx
+++ b/instruction_data/templates/dec_final/PIT_SI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/dec_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{855DE1A9-708D-2849-A42B-E1C1784A7D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF99D68-EBDC-0242-B117-306B03DEE6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="15520" xr2:uid="{810EA2B3-482B-894A-A620-1EEE84924FEB}"/>
   </bookViews>
@@ -17,10 +17,9 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PIT+SI payment'!$A$1:$E$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PIT+SI payment'!$A$1:$E$67</definedName>
     <definedName name="CHActCashBalance">#REF!</definedName>
     <definedName name="CHExpenseForcast">#REF!</definedName>
     <definedName name="CHFundrasingForcast">#REF!</definedName>
@@ -72,7 +71,7 @@
     <definedName name="YTDCashBalance">#REF!</definedName>
     <definedName name="YTDMonthOfCash">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -640,34 +639,6 @@
       <sheetData sheetId="27"/>
       <sheetData sheetId="28"/>
       <sheetData sheetId="29"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Transaction List with Splits"/>
-      <sheetName val="BS manual mapping"/>
-      <sheetName val="salary allocation-v2"/>
-      <sheetName val="PIT+SI payment (2)"/>
-      <sheetName val="30 Bank VN Vietnam (VND)"/>
-      <sheetName val="29 Bank VN Vietnam (USD)"/>
-      <sheetName val="34 Bank VN Vietnam (VND)"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1026,7 +997,7 @@
         <v>Amount</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>100</v>
       </c>
@@ -1035,7 +1006,7 @@
       <c r="D2" s="11"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>12</v>
       </c>
@@ -1052,7 +1023,7 @@
         <v>-15333896</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>12</v>
       </c>
@@ -1069,7 +1040,7 @@
         <v>-15483132</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>12</v>
       </c>
@@ -1086,7 +1057,7 @@
         <v>-15205906</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>12</v>
       </c>
@@ -1103,7 +1074,7 @@
         <v>-13970133</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
@@ -1120,7 +1091,7 @@
         <v>-8879531</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>12</v>
       </c>
@@ -1137,7 +1108,7 @@
         <v>-15316796</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>12</v>
       </c>
@@ -1154,7 +1125,7 @@
         <v>-6400558</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>12</v>
       </c>
@@ -1171,7 +1142,7 @@
         <v>-15117814</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>12</v>
       </c>
@@ -1188,7 +1159,7 @@
         <v>-15063924</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>12</v>
       </c>
@@ -1205,7 +1176,7 @@
         <v>-15117814</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>12</v>
       </c>
@@ -1222,7 +1193,7 @@
         <v>-14094497</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>12</v>
       </c>
@@ -1239,7 +1210,7 @@
         <v>-15534950</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>12</v>
       </c>
@@ -1256,7 +1227,7 @@
         <v>-3984832</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>12</v>
       </c>
@@ -1273,7 +1244,7 @@
         <v>-5064512</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
@@ -1290,7 +1261,7 @@
         <v>-6516352</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>12</v>
       </c>
@@ -1307,7 +1278,7 @@
         <v>-4564352</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>12</v>
       </c>
@@ -1324,7 +1295,7 @@
         <v>-5039552</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>12</v>
       </c>
@@ -1341,7 +1312,7 @@
         <v>-4069952</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>12</v>
       </c>
@@ -1358,7 +1329,7 @@
         <v>-4069952</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>12</v>
       </c>
@@ -1375,7 +1346,7 @@
         <v>-4564352</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>12</v>
       </c>
@@ -1392,7 +1363,7 @@
         <v>-4564352</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>12</v>
       </c>
@@ -1409,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>12</v>
       </c>
@@ -1426,7 +1397,7 @@
         <v>-3604352</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>12</v>
       </c>
@@ -1443,7 +1414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>12</v>
       </c>
@@ -1460,7 +1431,7 @@
         <v>-4160000</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>12</v>
       </c>
@@ -1477,7 +1448,7 @@
         <v>-1600000</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>12</v>
       </c>
@@ -1494,7 +1465,7 @@
         <v>-3976000</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>12</v>
       </c>
@@ -1511,7 +1482,7 @@
         <v>-4160000</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>12</v>
       </c>
@@ -1528,7 +1499,7 @@
         <v>-4160000</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>12</v>
       </c>
@@ -1545,347 +1516,333 @@
         <v>-4160000</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B33" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C33" s="11" t="s">
+    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D34" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="10">
+      <c r="E34" s="10">
         <v>-15333896</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C34" s="11" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D35" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="10">
+      <c r="E35" s="10">
         <v>-15483132</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B35" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C35" s="11" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C36" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D36" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E35" s="10">
+      <c r="E36" s="10">
         <v>-15205906</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C36" s="11" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D37" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E36" s="10">
+      <c r="E37" s="10">
         <v>-13970133</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B37" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C37" s="11" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C38" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D38" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="E37" s="10">
+      <c r="E38" s="10">
         <v>-8879531</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B38" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C38" s="11" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="D39" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E38" s="10">
+      <c r="E39" s="10">
         <v>-15316796</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C39" s="11" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C40" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D39" s="11" t="s">
+      <c r="D40" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="E39" s="10">
+      <c r="E40" s="10">
         <v>-6400558</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B40" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C40" s="11" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D41" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E40" s="10">
+      <c r="E41" s="10">
         <v>-15117814</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C41" s="11" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C42" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D42" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E41" s="10">
+      <c r="E42" s="10">
         <v>-15063924</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B42" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C42" s="11" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D43" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="10">
+      <c r="E43" s="10">
         <v>-15117814</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B43" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C43" s="11" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C44" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D44" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E43" s="10">
+      <c r="E44" s="10">
         <v>-14094497</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B44" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C44" s="11" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C45" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D45" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E44" s="10">
+      <c r="E45" s="10">
         <v>-15534950</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B45" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C45" s="11" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C46" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D46" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E45" s="10">
+      <c r="E46" s="10">
         <v>-3984832</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B46" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C46" s="11" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D47" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E46" s="10">
+      <c r="E47" s="10">
         <v>-5064512</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B47" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C47" s="11" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C48" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D48" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E47" s="10">
+      <c r="E48" s="10">
         <v>-6516352</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C48" s="11" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D48" s="11" t="s">
+      <c r="D49" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E48" s="10">
+      <c r="E49" s="10">
         <v>-4564352</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C49" s="11" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C50" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D50" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E49" s="10">
+      <c r="E50" s="10">
         <v>-5039552</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B50" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C50" s="11" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C51" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="D51" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E50" s="10">
+      <c r="E51" s="10">
         <v>-4069952</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B51" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C51" s="11" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C52" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D52" s="11" t="s">
         <v>29</v>
-      </c>
-      <c r="E51" s="10">
-        <v>-4564352</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B52" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D52" s="11" t="s">
-        <v>27</v>
       </c>
       <c r="E52" s="10">
         <v>-4564352</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="11" t="s">
         <v>12</v>
       </c>
@@ -1893,101 +1850,101 @@
         <v>46020</v>
       </c>
       <c r="C53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E53" s="10">
+        <v>-4564352</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C54" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D53" s="11" t="s">
+      <c r="D54" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E53" s="10">
+      <c r="E54" s="10">
         <v>-3604352</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B54" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C54" s="11" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D55" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E54" s="10">
+      <c r="E55" s="10">
         <v>-4160000</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C55" s="11" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C56" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D56" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E55" s="10">
+      <c r="E56" s="10">
         <v>-1600000</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B56" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C56" s="11" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C57" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D57" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E56" s="10">
+      <c r="E57" s="10">
         <v>-3976000</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B57" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C57" s="11" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C58" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D58" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="E57" s="10">
-        <v>-4160000</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B58" s="12">
-        <v>46020</v>
-      </c>
-      <c r="C58" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D58" s="11" t="s">
-        <v>15</v>
       </c>
       <c r="E58" s="10">
         <v>-4160000</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" s="11" t="s">
         <v>12</v>
       </c>
@@ -1995,16 +1952,16 @@
         <v>46020</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E59" s="10">
         <v>-4160000</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" s="11" t="s">
         <v>12</v>
       </c>
@@ -2012,42 +1969,42 @@
         <v>46020</v>
       </c>
       <c r="C60" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" s="10">
+        <v>-4160000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B61" s="12">
+        <v>46020</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="D61" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E60" s="10">
+      <c r="E61" s="10">
         <v>-5389074</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="6" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B61" s="5"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="3"/>
-    </row>
-    <row r="62" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B62" s="9">
-        <v>45999</v>
-      </c>
-      <c r="C62" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E62" s="7">
-        <v>-5703791</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="5"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" s="8" t="s">
         <v>4</v>
       </c>
@@ -2055,88 +2012,96 @@
         <v>45999</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E63" s="7">
-        <v>-960540</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+        <v>-5703791</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B64" s="9" t="s">
+      <c r="B64" s="9">
+        <v>45999</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E64" s="7">
+        <v>-960540</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="E65" s="1"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="C66" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D64" s="8" t="s">
+      <c r="D66" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E64" s="7">
+      <c r="E66" s="7">
         <v>-6000000</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="6" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="5"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="4"/>
-      <c r="E65" s="3"/>
-    </row>
-    <row r="73" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B67" s="5"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="3"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-    </row>
-    <row r="74" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-    </row>
-    <row r="75" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-    </row>
-    <row r="76" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-    </row>
-    <row r="77" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-    </row>
-    <row r="78" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-    </row>
-    <row r="79" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-    </row>
-    <row r="80" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-    </row>
-    <row r="81" spans="4:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-    </row>
-    <row r="82" spans="4:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-    </row>
-    <row r="83" spans="4:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-    </row>
-    <row r="84" spans="4:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E65" xr:uid="{CFE03B3B-C62C-4129-BB4A-082CF9BDF896}"/>

</xml_diff>